<commit_message>
[update] DropItem 및 player 상호 작용 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/WJUnit.xlsx
+++ b/JsonConverter/ExcelFiles/WJUnit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OZ_Project\WJMainProject2D\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB20FFA2-F3F6-4BE1-9655-FFBB144711EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3565D4B7-8137-4F99-A771-18C96DAA27BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29385" yWindow="3225" windowWidth="20370" windowHeight="11145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -584,7 +584,7 @@
         <v>9</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>21</v>

</xml_diff>